<commit_message>
results data and tables
</commit_message>
<xml_diff>
--- a/results_table.xlsx
+++ b/results_table.xlsx
@@ -13,21 +13,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="60" uniqueCount="37">
-  <si>
-    <t>Overall Score</t>
-  </si>
-  <si>
-    <t>N (%)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="65" uniqueCount="34">
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Overall Score (441 items per model)</t>
+  </si>
+  <si>
+    <t>n (%)</t>
   </si>
   <si>
     <t>95% CI</t>
   </si>
   <si>
-    <t>Other Items</t>
-  </si>
-  <si>
-    <t>Statistical Items</t>
+    <t>Other Items (315 items per model)</t>
+  </si>
+  <si>
+    <t>Statistical Items (126 items per model)</t>
   </si>
   <si>
     <t>Comparison: Descriptive vs Stats</t>
@@ -42,88 +45,76 @@
     <t>OpenAI GPT 5</t>
   </si>
   <si>
-    <t>331 (78%)</t>
-  </si>
-  <si>
-    <t>74% - 81%</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>242 (81%)</t>
-  </si>
-  <si>
-    <t>76% - 86%</t>
-  </si>
-  <si>
-    <t>89 (72%)</t>
-  </si>
-  <si>
-    <t>67% - 76%</t>
-  </si>
-  <si>
-    <t>0.16 (0.05 - 0.49)</t>
-  </si>
-  <si>
-    <t>0.001</t>
+    <t>343 (78%)</t>
+  </si>
+  <si>
+    <t>73% - 81%</t>
+  </si>
+  <si>
+    <t>263 (83%)</t>
+  </si>
+  <si>
+    <t>77% - 87%</t>
+  </si>
+  <si>
+    <t>80 (63%)</t>
+  </si>
+  <si>
+    <t>56% - 72%</t>
+  </si>
+  <si>
+    <t>0.10 (0.04 - 0.28)</t>
+  </si>
+  <si>
+    <t>&lt;0.001</t>
   </si>
   <si>
     <t>Google Gemini Pro</t>
   </si>
   <si>
-    <t>328 (77%)</t>
-  </si>
-  <si>
-    <t>74% - 80%</t>
-  </si>
-  <si>
-    <t>248 (83%)</t>
-  </si>
-  <si>
-    <t>78% - 88%</t>
-  </si>
-  <si>
-    <t>80 (67%)</t>
-  </si>
-  <si>
-    <t>60% - 73%</t>
-  </si>
-  <si>
-    <t>0.05 (0.02 - 0.16)</t>
-  </si>
-  <si>
-    <t>&lt;0.001</t>
+    <t>350 (79%)</t>
+  </si>
+  <si>
+    <t>74% - 82%</t>
+  </si>
+  <si>
+    <t>270 (86%)</t>
+  </si>
+  <si>
+    <t>80% - 89%</t>
+  </si>
+  <si>
+    <t>0.07 (0.03 - 0.20)</t>
   </si>
   <si>
     <t>Claude Sonnet</t>
   </si>
   <si>
-    <t>299 (78%)</t>
-  </si>
-  <si>
-    <t>222 (83%)</t>
-  </si>
-  <si>
-    <t>77% - 88%</t>
-  </si>
-  <si>
-    <t>77 (70%)</t>
-  </si>
-  <si>
-    <t>65% - 75%</t>
-  </si>
-  <si>
-    <t>0.10 (0.03 - 0.32)</t>
-  </si>
-  <si>
-    <t>0.79</t>
-  </si>
-  <si>
-    <t>0.66</t>
-  </si>
-  <si>
-    <t>0.13</t>
+    <t>352 (80%)</t>
+  </si>
+  <si>
+    <t>75% - 83%</t>
+  </si>
+  <si>
+    <t>89 (71%)</t>
+  </si>
+  <si>
+    <t>64% - 78%</t>
+  </si>
+  <si>
+    <t>0.21 (0.08 - 0.58)</t>
+  </si>
+  <si>
+    <t>0.003</t>
+  </si>
+  <si>
+    <t>0.51</t>
+  </si>
+  <si>
+    <t>0.46</t>
+  </si>
+  <si>
+    <t>0.12</t>
   </si>
 </sst>
 </file>
@@ -167,7 +158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -175,16 +166,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
         <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -192,16 +183,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -212,13 +203,13 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -229,30 +220,30 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -260,50 +251,50 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -311,33 +302,33 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -345,16 +336,16 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -362,15 +353,32 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
         <v>17</v>
       </c>
-      <c r="C12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>